<commit_message>
feat: keep only specified 8 home care topics
</commit_message>
<xml_diff>
--- a/public/stroke_links.xlsx
+++ b/public/stroke_links.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="EnrichedLinks" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,19 +418,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>S__83165253_0.jpg</v>
+        <v>S__83165254_0.jpg</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="str">
-        <v>ความรู้ทั่วไป</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D2" t="str">
-        <v>โรคหลอดเลือดสมองตีบ - Chulabhorn Channel</v>
+        <v>การให้อาหารทางสายยาง</v>
       </c>
       <c r="E2" t="str">
-        <v>https://chulabhornchannel.cra.ac.th/health-articles/23771/</v>
+        <v>https://youtube.com/playlist?list=PLVGq9IQHt11Zvao7gpzcZkFKVhLFSNgaT&amp;si=6iUzwzqeLeh9v6j0</v>
       </c>
     </row>
     <row r="3">
@@ -438,16 +438,16 @@
         <v>S__83165254_0.jpg</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C3" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D3" t="str">
-        <v>โภชนาการ</v>
+        <v>การวัดสัญญาณชีพ</v>
       </c>
       <c r="E3" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11YfUPZPPnnnvq4KgaWRY3ZF&amp;si=MS6MoIyjYTQzAGTG</v>
+        <v>https://youtube.com/playlist?list=PLVGq9IQHt11afju0DMzu5F5QjzOLB5Dp4&amp;si=Q18x1N_3hPCA0r_8</v>
       </c>
     </row>
     <row r="4">
@@ -455,16 +455,16 @@
         <v>S__83165254_0.jpg</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C4" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D4" t="str">
-        <v>การให้อาหารทางสายยาง</v>
+        <v>การเช็ดตัว และพลิกตัว</v>
       </c>
       <c r="E4" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11Zvao7gpzcZkFKVhLFSNgaT&amp;si=6iUzwzqeLeh9v6j0</v>
+        <v>https://youtube.com/playlist?list=PLVGq9IQHt11b78qVtVgcbz7L6CAekUDww&amp;si=QQqvVpgMT7AyCLXb</v>
       </c>
     </row>
     <row r="5">
@@ -472,16 +472,16 @@
         <v>S__83165254_0.jpg</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C5" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D5" t="str">
-        <v>คู่มือการเตรียมความพร้อมในการดูแลผู้ป่ว.pdf</v>
+        <v>การใช้เตียงและที่นอนลม</v>
       </c>
       <c r="E5" t="str">
-        <v>https://drive.google.com/file/d/1JdzU-8qLQNBqfkcLclKQp5OOHJpjqp8F/view?usp=drive_link</v>
+        <v>https://youtube.com/playlist?list=PLVGq9IQHt11YayUXVvKil01jSxjv6a5Ok&amp;si=bEhMsbfCv5fn5Sjc</v>
       </c>
     </row>
     <row r="6">
@@ -489,16 +489,16 @@
         <v>S__83165254_0.jpg</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C6" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D6" t="str">
-        <v>การดูแลประคับประคอง</v>
+        <v>การให้ออกซิเจน</v>
       </c>
       <c r="E6" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11bLanp3R3L8xys9iCyCzH2K&amp;si=elzFhpAHBPe4DRiU</v>
+        <v>https://youtube.com/playlist?list=PLVGq9IQHt11YLl4U_IpwPKqcL3LT_tjW-&amp;si=Ka8yzDUThkLanPnQ</v>
       </c>
     </row>
     <row r="7">
@@ -506,16 +506,16 @@
         <v>S__83165254_0.jpg</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C7" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D7" t="str">
-        <v>การทำแผลกดทับ</v>
+        <v>วิธีการดูดเสมหะ</v>
       </c>
       <c r="E7" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11YeP8lyyTyCo6seXqn6CUpV&amp;si=WvRwyc6UE6tOggoO</v>
+        <v>https://youtube.com/playlist?list=PLVGq9IQHt11afzRK0rwB4AmDQBxFcTRys&amp;si=tIhiedllv-tQ7Lcu</v>
       </c>
     </row>
     <row r="8">
@@ -523,16 +523,16 @@
         <v>S__83165254_0.jpg</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C8" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D8" t="str">
-        <v>การใช้เตียงและที่นอนลม</v>
+        <v>การดูแลท่อหลอดลมคอ</v>
       </c>
       <c r="E8" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11YayUXVvKil01jSxjv6a5Ok&amp;si=bEhMsbfCv5fn5Sjc</v>
+        <v>https://youtube.com/playlist?list=PLVGq9IQHt11Y9yoKfhS4dSUpN1e1ZZt74&amp;si=445_8vwMvqhpqg83</v>
       </c>
     </row>
     <row r="9">
@@ -540,191 +540,21 @@
         <v>S__83165254_0.jpg</v>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C9" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
+        <v>คู่มือการดูแลผู้ป่วยที่บ้าน</v>
       </c>
       <c r="D9" t="str">
-        <v>การวัดสัญญาณชีพ</v>
+        <v>การดูแลสายสวนปัสสาวะ</v>
       </c>
       <c r="E9" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11afju0DMzu5F5QjzOLB5Dp4&amp;si=Q18x1N_3hPCA0r_8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B10">
-        <v>8</v>
-      </c>
-      <c r="C10" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D10" t="str">
-        <v>การเช็ดตัว และพลิกตัว</v>
-      </c>
-      <c r="E10" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11b78qVtVgcbz7L6CAekUDww&amp;si=QQqvVpgMT7AyCLXb</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B11">
-        <v>9</v>
-      </c>
-      <c r="C11" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D11" t="str">
-        <v>วิธีการดูดเสมหะ</v>
-      </c>
-      <c r="E11" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11afzRK0rwB4AmDQBxFcTRys&amp;si=tIhiedllv-tQ7Lcu</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B12">
-        <v>10</v>
-      </c>
-      <c r="C12" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D12" t="str">
-        <v>การให้ออกซิเจน</v>
-      </c>
-      <c r="E12" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11YLl4U_IpwPKqcL3LT_tjW-&amp;si=Ka8yzDUThkLanPnQ</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B13">
-        <v>11</v>
-      </c>
-      <c r="C13" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D13" t="str">
-        <v>การดูแลท่อหลอดลมคอ</v>
-      </c>
-      <c r="E13" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11Y9yoKfhS4dSUpN1e1ZZt74&amp;si=445_8vwMvqhpqg83</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B14">
-        <v>12</v>
-      </c>
-      <c r="C14" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D14" t="str">
-        <v>การฉีดยาเข้าใต้ผิวหนัง</v>
-      </c>
-      <c r="E14" t="str">
         <v>https://youtube.com/playlist?list=PLVGq9IQHt11Zd7NBo3Ay9Vi74D5cNXBFj&amp;si=FTLMfwKKRlSXXIuq</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B15">
-        <v>13</v>
-      </c>
-      <c r="C15" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D15" t="str">
-        <v>ความรู้เรื่องโรคมะเร็ง</v>
-      </c>
-      <c r="E15" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11aGhVsJJmEkuCUd6DkqTBdl&amp;si=-stsylHTcYMxkkNB</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B16">
-        <v>14</v>
-      </c>
-      <c r="C16" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D16" t="str">
-        <v>การออกกำลังกาย</v>
-      </c>
-      <c r="E16" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11YzYKDnNuS7qYK-niNN59YU&amp;si=n_iFbL7jdR6LCroy</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>S__83165254_0.jpg</v>
-      </c>
-      <c r="B17">
-        <v>15</v>
-      </c>
-      <c r="C17" t="str">
-        <v>การดูแลผู้ป่วยที่บ้าน</v>
-      </c>
-      <c r="D17" t="str">
-        <v>ดูแลใจผู้ดูแล</v>
-      </c>
-      <c r="E17" t="str">
-        <v>https://youtube.com/playlist?list=PLVGq9IQHt11b27XwxpuTQntsIZo_jRVnz&amp;si=r5u6OzBBh-k9ubKT</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>S__83165255_0.jpg</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18" t="str">
-        <v>แบบประเมิน</v>
-      </c>
-      <c r="D18" t="str">
-        <v>แบบประเมินความพึงพอใจการดูแลผู้ป่วย</v>
-      </c>
-      <c r="E18" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdv-5PwGv9IG3jLP_3kQnrkkp36GvG6sCx_9OSgwhyOj3GjnA/viewform</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>S__83165256_0.jpg</v>
-      </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
-      <c r="C19" t="str">
-        <v>กายภาพบำบัด</v>
-      </c>
-      <c r="D19" t="str">
-        <v>การกายภาพเบื้องต้นสำหรับผู้ป่วยอัมพาตใบหน้าครึ่งซีก (Bell’s palsy)</v>
-      </c>
-      <c r="E19" t="str">
-        <v>https://youtu.be/Vh_Qo3JPfQ4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: keep 8 home care topics plus evaluation form link (9 items total)
</commit_message>
<xml_diff>
--- a/public/stroke_links.xlsx
+++ b/public/stroke_links.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -552,9 +552,26 @@
         <v>https://youtube.com/playlist?list=PLVGq9IQHt11Zd7NBo3Ay9Vi74D5cNXBFj&amp;si=FTLMfwKKRlSXXIuq</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>S__83165255_0.jpg</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>แบบประเมิน</v>
+      </c>
+      <c r="D10" t="str">
+        <v>แบบประเมินความพึงพอใจการดูแลผู้ป่วย</v>
+      </c>
+      <c r="E10" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdv-5PwGv9IG3jLP_3kQnrkkp36GvG6sCx_9OSgwhyOj3GjnA/viewform</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>